<commit_message>
update 20 de Mayo con datos previos. Ajuste texto
</commit_message>
<xml_diff>
--- a/mad-map-data-v2.xlsx
+++ b/mad-map-data-v2.xlsx
@@ -646,7 +646,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="16" customHeight="1" s="24">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -750,7 +749,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="16" customHeight="1" s="24">
       <c r="A14" s="26" t="inlineStr">
         <is>
@@ -2912,7 +2910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="24" min="1" max="1"/>
@@ -7150,7 +7148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="24" min="1" max="1"/>
@@ -7170,7 +7168,7 @@
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Área principal es lectura — un investigador puede operar en varias. Profundización en 12_Investigador_Lab y 13_Investigador_Modo.</t>
+          <t>Área principal es lectura — un investigador puede operar en varias. área_secundaria: segunda área autodeclarada (formulario 2024). perfil_anid desde formulario 2024; orcid y google_scholar: pendiente completar. Nota: URL ANID de Di Felice en formulario era inválida — celda vacía, pendiente corregir.</t>
         </is>
       </c>
     </row>
@@ -7192,10 +7190,30 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
+          <t>área_secundaria</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
           <t>perfil_casiopea</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>perfil_anid</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>perfil_orcid</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>perfil_google_scholar</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>estado_perfil</t>
         </is>
@@ -7217,12 +7235,18 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Ursula_Exss</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://investigadores.anid.cl/es/public_search/researcher?id=38268</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>consolidado Casiopea + ANID</t>
         </is>
@@ -7244,12 +7268,18 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Katherine_Exss</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://investigadores.anid.cl/es/public_search/researcher?id=39442</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>consolidado Casiopea + ANID</t>
         </is>
@@ -7271,12 +7301,13 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Jorge_Ferrada</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>bio + cursos + proyectos + tesis</t>
         </is>
@@ -7300,10 +7331,15 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
+          <t>FCT</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
           <t>https://wiki.ead.pucv.cl/Andr%C3%A9s_Garc%C3%A9s</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>línea explícita</t>
         </is>
@@ -7325,12 +7361,13 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Iv%C3%A1n_Ivelic</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>línea explícita + lectura detallada</t>
         </is>
@@ -7352,12 +7389,13 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/David_Luza</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>consolidado Casiopea + ANID</t>
         </is>
@@ -7379,12 +7417,13 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Adriana_Mar%C3%ADn</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>líneas explícitas</t>
         </is>
@@ -7406,12 +7445,13 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/%C3%81lvaro_Mercado</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>líneas explícitas</t>
         </is>
@@ -7433,12 +7473,18 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Jaime_Reyes</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://investigadores.anid.cl/es/public_search/researcher?id=44715</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>tema/área explícita</t>
         </is>
@@ -7460,12 +7506,18 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Rodrigo_Saavedra</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://investigadores.anid.cl/es/public_search/researcher?id=36228</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>líneas explícitas</t>
         </is>
@@ -7489,10 +7541,20 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
+          <t>ECH</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
           <t>https://wiki.ead.pucv.cl/Daniela_Salgado</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://investigadores.anid.cl/es/public_search/researcher?id=43532</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>líneas explícitas</t>
         </is>
@@ -7514,12 +7576,18 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Herbert_Spencer</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://investigadores.anid.cl/es/public_search/researcher?id=6662</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>líneas explícitas</t>
         </is>
@@ -7541,12 +7609,13 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Alfred_Thiers</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>líneas explícitas</t>
         </is>
@@ -7568,12 +7637,13 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Lorena_Herrera</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>ANID</t>
         </is>
@@ -7595,12 +7665,13 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Juan_Carlos_Jeldes</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>lectura detallada de perfil</t>
         </is>
@@ -7622,12 +7693,13 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Mich%C3%A8le_Wilkomirsky</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>ANID</t>
         </is>
@@ -7651,10 +7723,20 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
+          <t>ECH</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
           <t>https://wiki.ead.pucv.cl/%C3%93scar_Andrade</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://investigadores.anid.cl/es/public_search/researcher?id=41600</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>ANID</t>
         </is>
@@ -7678,10 +7760,20 @@
       </c>
       <c r="D22" s="21" t="inlineStr">
         <is>
+          <t>ECH</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
           <t>https://wiki.ead.pucv.cl/Anna_Braghini</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://investigadores.anid.cl/es/people/49354-Anna_Braghini</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>deducción razonable</t>
         </is>
@@ -7703,12 +7795,13 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Arturo_Chicano</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>lectura detallada de perfil</t>
         </is>
@@ -7730,12 +7823,13 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Sylvia_Arriagada</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>línea explícita + lectura detallada</t>
         </is>
@@ -7757,12 +7851,13 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Marcelo_Araya</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>deducción fundada</t>
         </is>
@@ -7786,10 +7881,15 @@
       </c>
       <c r="D26" s="21" t="inlineStr">
         <is>
+          <t>EAA</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
           <t>https://wiki.ead.pucv.cl/Emanuela_Di_Felice</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>consolidado por lectura detallada</t>
         </is>
@@ -7797,8 +7897,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId1"/>

</xml_diff>

<commit_message>
ajustes de datos. campos nuevos
</commit_message>
<xml_diff>
--- a/mad-map-data-v2.xlsx
+++ b/mad-map-data-v2.xlsx
@@ -7168,7 +7168,7 @@
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
         <is>
-          <t>Área principal es lectura — un investigador puede operar en varias. área_secundaria: segunda área autodeclarada (formulario 2024). perfil_anid desde formulario 2024; orcid y google_scholar: pendiente completar. Nota: URL ANID de Di Felice en formulario era inválida — celda vacía, pendiente corregir.</t>
+          <t>Área principal es lectura — un investigador puede operar en varias. área_secundaria: segunda área autodeclarada (formulario 2024). perfil_anid desde formulario 2024; orcid y google_scholar: pendiente completar. Nota: URL ANID de Emanuela Di Felice en formulario era inválida — vacía, pendiente corregir.</t>
         </is>
       </c>
     </row>
@@ -7193,7 +7193,7 @@
           <t>área_secundaria</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>perfil_casiopea</t>
         </is>
@@ -7235,8 +7235,7 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Ursula_Exss</t>
         </is>
@@ -7268,8 +7267,7 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Katherine_Exss</t>
         </is>
@@ -7301,8 +7299,7 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Jorge_Ferrada</t>
         </is>
@@ -7329,12 +7326,12 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>FCT</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Andr%C3%A9s_Garc%C3%A9s</t>
         </is>
@@ -7361,8 +7358,7 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Iv%C3%A1n_Ivelic</t>
         </is>
@@ -7389,8 +7385,7 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/David_Luza</t>
         </is>
@@ -7417,8 +7412,7 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Adriana_Mar%C3%ADn</t>
         </is>
@@ -7445,8 +7439,7 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/%C3%81lvaro_Mercado</t>
         </is>
@@ -7473,8 +7466,7 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Jaime_Reyes</t>
         </is>
@@ -7506,8 +7498,7 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Rodrigo_Saavedra</t>
         </is>
@@ -7539,12 +7530,12 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>ECH</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Daniela_Salgado</t>
         </is>
@@ -7576,8 +7567,7 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Herbert_Spencer</t>
         </is>
@@ -7609,8 +7599,7 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Alfred_Thiers</t>
         </is>
@@ -7637,8 +7626,7 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D18" s="21" t="n"/>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Lorena_Herrera</t>
         </is>
@@ -7665,8 +7653,7 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Juan_Carlos_Jeldes</t>
         </is>
@@ -7693,8 +7680,7 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Mich%C3%A8le_Wilkomirsky</t>
         </is>
@@ -7721,12 +7707,12 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>ECH</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/%C3%93scar_Andrade</t>
         </is>
@@ -7758,12 +7744,12 @@
           <t>EAA</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>ECH</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Anna_Braghini</t>
         </is>
@@ -7795,8 +7781,7 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Arturo_Chicano</t>
         </is>
@@ -7823,8 +7808,7 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Sylvia_Arriagada</t>
         </is>
@@ -7851,8 +7835,7 @@
           <t>FCT</t>
         </is>
       </c>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Marcelo_Araya</t>
         </is>
@@ -7879,12 +7862,12 @@
           <t>ECH</t>
         </is>
       </c>
-      <c r="D26" s="21" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>EAA</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>https://wiki.ead.pucv.cl/Emanuela_Di_Felice</t>
         </is>
@@ -7900,11 +7883,6 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId3"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>